<commit_message>
docs: thêm phiếu giao việc chi tiết cho task khởi động Phase 0
- docs/tasks/README.md: khung 7 mục cho phiếu giao việc.
- docs/tasks/phase-0-starters.md: phiếu chi tiết CT1, IN1, FE1
  (mục tiêu, bối cảnh, từng bước có file/lệnh cụ thể, DoD, cách kiểm tra,
  docs liên quan, nhánh & PR) để thành viên biết bắt đầu từ đâu.
- Kế hoạch (xlsx): trỏ CT1/IN1/FE1 tới phiếu chi tiết ở cột note/Gợi ý;
  thêm dòng "Phiếu giao việc chi tiết" vào Quy ước & Điều phối.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -665,7 +665,11 @@
       <c r="H3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -702,7 +706,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>ci.yml chạy pnpm check trên mọi PR + cache pnpm đã có; còn bật branch protection main + tạo PR mẫu</t>
+          <t>ci.yml chạy pnpm check trên mọi PR + cache pnpm đã có; còn bật branch protection main + tạo PR mẫu · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -739,7 +743,11 @@
       <c r="H5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -3128,7 +3136,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>docs/06; .github/workflows/ci.yml</t>
+          <t>docs/06; .github/workflows/ci.yml · 📄 Phiếu chi tiết: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3188,7 +3196,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>docs/04 §3.2 (URL tiếng Anh); Navbar/SiteFooter có sẵn</t>
+          <t>docs/04 §3.2 (URL tiếng Anh); Navbar/SiteFooter có sẵn · 📄 Phiếu chi tiết: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3248,7 +3256,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>docs/08 §2; chặn công bố</t>
+          <t>docs/08 §2; chặn công bố · 📄 Phiếu chi tiết: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -11582,7 +11590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11660,58 +11668,70 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Cách dùng sheet</t>
+          <t>Phiếu giao việc chi tiết</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Bảng nhiệm vụ = backlog tổng (lọc theo Ưu tiên/Phase/Phụ trách). Backend/Frontend/Hạ tầng &amp; QA/Nội dung &amp; Docs = task con theo mảng — mỗi bạn mở sheet mảng của mình. Thành viên = ai làm gì. Ưu tiên/Trạng thái có dropdown và tự tô màu.</t>
+          <t>Mỗi task có phiếu chi tiết ở docs/tasks/*.md (bối cảnh, file cụ thể, từng bước, lệnh, Định nghĩa Hoàn thành, cách kiểm tra). Bắt đầu: docs/tasks/phase-0-starters.md (CT1, IN1, FE1). Task chưa có phiếu thì copy khung 7 mục trong docs/tasks/README.md.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Thứ tự ưu tiên</t>
+          <t>Cách dùng sheet</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Làm P0 trước, rồi P1, rồi P2. Không bắt đầu task khi 'Phụ thuộc' chưa Xong (vd chưa có BE1 thì khoan làm BE5).</t>
+          <t>Lộ trình = bảng cả nhóm cùng đọc từ trên xuống &amp; tick. Bảng nhiệm vụ = backlog tổng (lọc theo Ưu tiên/Phase/Phụ trách). Backend/Frontend/Hạ tầng &amp; QA/Nội dung &amp; Docs = task con theo mảng — mỗi bạn mở sheet mảng của mình. Thành viên = ai làm gì. Ưu tiên/Trạng thái có dropdown và tự tô màu.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Timeline</t>
+          <t>Thứ tự ưu tiên</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CHƯA chốt deadline — cột Deadline để trống, trưởng dự án tự chia theo Phase. Gợi ý: Phase 0 (nền tảng) → Phase 1 (website + tuyển) → Phase 2 (portal + quản trị + 2FA + audit). Scope đã ~2.5x so với bản đầu; cân nguồn lực trước khi đặt mốc.</t>
+          <t>Làm P0 trước, rồi P1, rồi P2. Không bắt đầu task khi 'Phụ thuộc' chưa Xong (vd chưa có BE1 thì khoan làm BE5).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Nhịp làm việc</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Check-in ngắn 15' hai lần/tuần. Trước mỗi buổi tự cập nhật Trạng thái + Tiến độ + Ghi chú.</t>
+          <t>CHƯA chốt deadline — cột Deadline để trống, trưởng dự án tự chia theo Phase. Gợi ý: Phase 0 (nền tảng) → Phase 1 (website + tuyển) → Phase 2 (portal + quản trị + 2FA + audit). Scope đã ~2.5x so với bản đầu; cân nguồn lực trước khi đặt mốc.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
+          <t>Nhịp làm việc</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Check-in ngắn 15' hai lần/tuần. Trước mỗi buổi tự cập nhật Trạng thái + Tiến độ + Ghi chú.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
           <t>Khi bị kẹt (Blocked)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Kẹt quá nửa ngày → Trạng thái=Blocked, ghi lý do, báo nhóm ngay. Không im lặng ôm task.</t>
         </is>

</xml_diff>

<commit_message>
chore(plan): FE1 chuyển Review (PR #1); đánh dấu subtask FE1 xong
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -737,15 +737,15 @@
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+          <t>PR #1 chờ review/merge: github.com/GrootTheDeveloper/apc-portal/pull/1 · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -3216,11 +3216,11 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="K5" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
@@ -9148,7 +9148,11 @@
           <t>0.5h</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -9232,7 +9236,11 @@
           <t>1h</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -9260,7 +9268,11 @@
           <t>1h</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore(plan): FE1 Xong (merged PR #1); IN1 70% (còn branch protection)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -702,11 +702,11 @@
         </is>
       </c>
       <c r="H4" s="3" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>ci.yml chạy pnpm check trên mọi PR + cache pnpm đã có; còn bật branch protection main + tạo PR mẫu · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+          <t>ci.yml + cache pnpm ✓; PR #1 đã xác nhận CI chạy trên PR ✓; CÒN LẠI: bật branch protection main · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
@@ -745,7 +745,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>PR #1 chờ review/merge: github.com/GrootTheDeveloper/apc-portal/pull/1 · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+          <t>Đã merge PR #1 vào main · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="K4" s="3" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="n">

</xml_diff>

<commit_message>
chore: CT1 gói trình duyệt + trạng thái IN1/CT1
- docs/tasks/ct1-review-package.md: gói trình APC duyệt trang chủ
  (cách demo, thay đổi vs bản gốc, nội dung mẫu cần thay, checklist chốt).
- Plan: CT1 → Đang làm (gói sẵn, chờ APC); IN1 → 80% (branch protection
  bị chặn do repo private trên GitHub Free — cần Pro hoặc public).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -659,15 +659,15 @@
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+          <t>Gói trình duyệt sẵn: docs/tasks/ct1-review-package.md. Chờ APC duyệt + cấp số liệu CLB/đối tác thật. · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -702,11 +702,11 @@
         </is>
       </c>
       <c r="H4" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>ci.yml + cache pnpm ✓; PR #1 đã xác nhận CI chạy trên PR ✓; CÒN LẠI: bật branch protection main · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+          <t>ci.yml + cache + PR mẫu (PR #1) ✓. Branch protection CHƯA bật được: repo private trên GitHub Free cần nâng Pro HOẶC để repo public. Tạm dùng quy ước PR + CI (chưa enforce). · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="K4" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
@@ -3276,11 +3276,11 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(plan): IN1 Xong — branch protection đã bật (repo public)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -698,15 +698,15 @@
       <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H4" s="3" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>ci.yml + cache + PR mẫu (PR #1) ✓. Branch protection CHƯA bật được: repo private trên GitHub Free cần nâng Pro HOẶC để repo public. Tạm dùng quy ước PR + CI (chưa enforce). · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+          <t>Branch protection đã bật (repo public): PR bắt buộc + 1 review + CI 'quality' xanh + up-to-date. enforce_admins=false (admin bypass khi cần). · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -3156,11 +3156,11 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K4" s="3" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(plan): CT1 Xong — trang chủ redesign đã duyệt (05/09/2026)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -659,15 +659,15 @@
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H3" s="3" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Gói trình duyệt sẵn: docs/tasks/ct1-review-package.md. Chờ APC duyệt + cấp số liệu CLB/đối tác thật. · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
+          <t>Đã duyệt 05/09/2026 (trưởng dự án); trang chủ redesign được công bố. Cấp số liệu CLB/đối tác thật chuyển sang CT2. · 📄 Phiếu: docs/tasks/phase-0-starters.md</t>
         </is>
       </c>
     </row>
@@ -3276,11 +3276,11 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: ghi nhận ORM=Prisma; BE1 vào review (PR #2); ghi chú BE-REC1
- docs/06-architecture.md: chốt ORM = Prisma cho BE1.
- Plan: BE1 → Review (PR #2 của HoangThienPD, chờ sửa 2 điểm review + approve);
  BE-REC1 ghi chú bổ sung model RecruitmentQuestion (BE1 đã có RecruitmentRound).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -776,13 +776,17 @@
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="4" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>PR #2 (branch feat/be1-db-schema, HoangThienPD): schema + migration Prisma. Chờ sửa 2 điểm review (script --schema, gitignore generated) + approve.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -3036,11 +3040,11 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
@@ -4636,7 +4640,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>docs/03 FLOW-06; sitemap PAGE-MGT-REC</t>
+          <t>docs/03 FLOW-06; sitemap PAGE-MGT-REC · ⚠️ BE1 đã có RecruitmentRound + application (PR #2); BE-REC1 bổ sung model RecruitmentQuestion.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore(plan): BE1 Xong — merged PR #2 (DB schema Prisma)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -776,15 +776,15 @@
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H6" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>PR #2 (branch feat/be1-db-schema, HoangThienPD): schema + migration Prisma. Chờ sửa 2 điểm review (script --schema, gitignore generated) + approve.</t>
+          <t>Đã merge PR #2 vào main (05/09/2026): schema Prisma + migration init (user, department, post, event, project, recruitment_round, application) + ERD. Fix review đã áp (script --schema, gitignore generated/).</t>
         </is>
       </c>
     </row>
@@ -3040,11 +3040,11 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(plan): bổ sung tên thành viên vào 9 pod + cột Phụ trách
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -83,7 +83,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -105,11 +105,55 @@
         <color rgb="00D0D5DD"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D5DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D5DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -136,6 +180,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -631,6 +677,14 @@
           <t>PHASE 0 · Nền tảng — làm trước tiên, mở đường cho mọi thứ</t>
         </is>
       </c>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="10" t="n"/>
+      <c r="H2" s="10" t="n"/>
+      <c r="I2" s="11" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -687,7 +741,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>OP-1</t>
+          <t>OP-1 · Đặng Phúc An Khang</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -726,7 +780,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -765,7 +819,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -804,7 +858,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -839,7 +893,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -874,7 +928,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -909,7 +963,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -934,6 +988,14 @@
           <t>PHASE 1 · Website công khai + Tuyển thành viên</t>
         </is>
       </c>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
+      <c r="H11" s="10" t="n"/>
+      <c r="I11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -951,7 +1013,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -986,7 +1048,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1021,7 +1083,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1056,7 +1118,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1091,7 +1153,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1126,7 +1188,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1161,7 +1223,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1196,7 +1258,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1231,7 +1293,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1266,7 +1328,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1301,7 +1363,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1336,7 +1398,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1371,7 +1433,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1406,7 +1468,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1441,7 +1503,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1476,7 +1538,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1501,6 +1563,14 @@
           <t>PHASE 2 · Portal thành viên + Quản trị + Bảo mật</t>
         </is>
       </c>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="10" t="n"/>
+      <c r="I28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1518,7 +1588,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1553,7 +1623,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1588,7 +1658,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1623,7 +1693,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -1658,7 +1728,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1693,7 +1763,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -1728,7 +1798,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -1763,7 +1833,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -1798,7 +1868,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -1833,7 +1903,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -1868,7 +1938,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -1903,7 +1973,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -1938,7 +2008,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -1973,7 +2043,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -2008,7 +2078,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -2043,7 +2113,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -2078,7 +2148,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -2113,7 +2183,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2148,7 +2218,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -2183,7 +2253,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -2218,7 +2288,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -2253,7 +2323,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -2288,7 +2358,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -2323,7 +2393,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
@@ -2358,7 +2428,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -2393,7 +2463,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -2428,7 +2498,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -2463,7 +2533,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -2498,7 +2568,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -2533,7 +2603,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -2568,7 +2638,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -2603,7 +2673,7 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -2638,7 +2708,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>OP-1</t>
+          <t>OP-1 · Đặng Phúc An Khang</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
@@ -2673,7 +2743,7 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>OP-1</t>
+          <t>OP-1 · Đặng Phúc An Khang</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -2708,7 +2778,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>OP-2</t>
+          <t>OP-2 · Nguyễn Tiến Bảo</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
@@ -2733,6 +2803,14 @@
           <t>LIÊN TỤC · Làm song song suốt dự án</t>
         </is>
       </c>
+      <c r="B64" s="10" t="n"/>
+      <c r="C64" s="10" t="n"/>
+      <c r="D64" s="10" t="n"/>
+      <c r="E64" s="10" t="n"/>
+      <c r="F64" s="10" t="n"/>
+      <c r="G64" s="10" t="n"/>
+      <c r="H64" s="10" t="n"/>
+      <c r="I64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -2750,7 +2828,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
@@ -2785,7 +2863,7 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -2820,7 +2898,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>OP-2</t>
+          <t>OP-2 · Nguyễn Tiến Bảo</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
@@ -2855,7 +2933,7 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>OP-2</t>
+          <t>OP-2 · Nguyễn Tiến Bảo</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -3025,7 +3103,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -3085,7 +3163,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -3145,7 +3223,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>OP-1</t>
+          <t>OP-1 · Đặng Phúc An Khang</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -3205,7 +3283,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -3325,7 +3403,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -3385,7 +3463,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -3445,7 +3523,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -3505,7 +3583,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -3565,7 +3643,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -3625,7 +3703,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -3685,7 +3763,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -3745,7 +3823,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -3805,7 +3883,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>FE-1</t>
+          <t>FE-1 · Lương Huỳnh</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -3865,7 +3943,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -3925,7 +4003,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -3985,7 +4063,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -4045,7 +4123,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -4105,7 +4183,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -4165,7 +4243,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -4225,7 +4303,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -4285,7 +4363,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -4345,7 +4423,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -4405,7 +4483,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -4465,7 +4543,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -4525,7 +4603,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -4585,7 +4663,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -4645,7 +4723,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -4705,7 +4783,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -4765,7 +4843,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -4825,7 +4903,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -4885,7 +4963,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -4945,7 +5023,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>FE-2</t>
+          <t>FE-2 · Nguyễn Gia Bảo</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -5005,7 +5083,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -5065,7 +5143,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -5125,7 +5203,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -5185,7 +5263,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -5245,7 +5323,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -5305,7 +5383,7 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -5365,7 +5443,7 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -5425,7 +5503,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -5485,7 +5563,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -5545,7 +5623,7 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -5605,7 +5683,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -5665,7 +5743,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>BE-3</t>
+          <t>BE-3 · Phan Anh Khương</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -5725,7 +5803,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -5785,7 +5863,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>BE-1</t>
+          <t>BE-1 · Phạm Đăng Hoàng Thiên</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -5845,7 +5923,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -5905,7 +5983,7 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -5965,7 +6043,7 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>BE-2</t>
+          <t>BE-2 · Trương Phúc Minh</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
@@ -6025,7 +6103,7 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
@@ -6085,7 +6163,7 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
@@ -6145,7 +6223,7 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
@@ -6205,7 +6283,7 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
@@ -6265,7 +6343,7 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
@@ -6325,7 +6403,7 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
@@ -6385,7 +6463,7 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>FE-3</t>
+          <t>FE-3 · Lê Đăng Nghĩa</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
@@ -6445,7 +6523,7 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>OP-1</t>
+          <t>OP-1 · Đặng Phúc An Khang</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
@@ -6505,7 +6583,7 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>OP-1</t>
+          <t>OP-1 · Đặng Phúc An Khang</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
@@ -6565,7 +6643,7 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>OP-2</t>
+          <t>OP-2 · Nguyễn Tiến Bảo</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
@@ -6625,7 +6703,7 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>FE-4</t>
+          <t>FE-4 · Huỳnh Hoàn Phúc</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
@@ -6685,7 +6763,7 @@
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>OP-2</t>
+          <t>OP-2 · Nguyễn Tiến Bảo</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
@@ -6745,7 +6823,7 @@
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>OP-2</t>
+          <t>OP-2 · Nguyễn Tiến Bảo</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
@@ -11333,7 +11411,11 @@
           <t>BE-1</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Phạm Đăng Hoàng Thiên</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Backend</t>
@@ -11362,7 +11444,11 @@
           <t>BE-2</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Trương Phúc Minh</t>
+        </is>
+      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Backend</t>
@@ -11391,7 +11477,11 @@
           <t>BE-3</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Phan Anh Khương</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Backend</t>
@@ -11420,7 +11510,11 @@
           <t>FE-1</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Lương Huỳnh</t>
+        </is>
+      </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -11449,7 +11543,11 @@
           <t>FE-2</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Nguyễn Gia Bảo</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -11478,7 +11576,11 @@
           <t>FE-3</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Lê Đăng Nghĩa</t>
+        </is>
+      </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -11507,7 +11609,11 @@
           <t>FE-4</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Huỳnh Hoàn Phúc</t>
+        </is>
+      </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -11536,7 +11642,11 @@
           <t>OP-1</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Đặng Phúc An Khang</t>
+        </is>
+      </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Hạ tầng/QA</t>
@@ -11565,7 +11675,11 @@
           <t>OP-2</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Nguyễn Tiến Bảo</t>
+        </is>
+      </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Hạ tầng/QA</t>
@@ -11588,6 +11702,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(tasks): phiếu Wave 1 (BE4, BE3, BE2, FE2, website mock) + link vào plan
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APC-Portal-Ke-hoach-cong-viec.xlsx
+++ b/APC-Portal-Ke-hoach-cong-viec.xlsx
@@ -875,7 +875,11 @@
       <c r="H7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/wave-1-p1.md</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -910,7 +914,11 @@
       <c r="H8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/wave-1-p1.md</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -945,7 +953,11 @@
       <c r="H9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/wave-1-p1.md</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -980,7 +992,11 @@
       <c r="H10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/wave-1-p1.md</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1380,7 +1396,11 @@
       <c r="H22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/wave-1-p1.md</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1415,7 +1435,11 @@
       <c r="H23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/wave-1-p1.md</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1450,7 +1474,11 @@
       <c r="H24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>📄 Phiếu: docs/tasks/wave-1-p1.md</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -3158,7 +3186,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Mật khẩu admin trong .env, KHÔNG hardcode</t>
+          <t>Mật khẩu admin trong .env, KHÔNG hardcode · 📄 Phiếu: docs/tasks/wave-1-p1.md</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3458,7 +3486,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>docs/03 FLOW-10; validate bằng Zod</t>
+          <t>docs/03 FLOW-10; validate bằng Zod · 📄 Phiếu: docs/tasks/wave-1-p1.md</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3578,7 +3606,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>docs/02 là nguồn chuẩn</t>
+          <t>docs/02 là nguồn chuẩn · 📄 Phiếu: docs/tasks/wave-1-p1.md</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3758,7 +3786,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>dùng Button có sẵn; gọi /auth (BE3)</t>
+          <t>dùng Button có sẵn; gọi /auth (BE3) · 📄 Phiếu: docs/tasks/wave-1-p1.md</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -4358,7 +4386,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>tái dùng NewsSection</t>
+          <t>tái dùng NewsSection · 📄 Phiếu: docs/tasks/wave-1-p1.md</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -4418,7 +4446,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>docs/03 FLOW-14; tái dùng EventsSection</t>
+          <t>docs/03 FLOW-14; tái dùng EventsSection · 📄 Phiếu: docs/tasks/wave-1-p1.md</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -4478,7 +4506,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>tái dùng bố cục ProjectsSection</t>
+          <t>tái dùng bố cục ProjectsSection · 📄 Phiếu: docs/tasks/wave-1-p1.md</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -11702,7 +11730,6 @@
       </c>
       <c r="G10" s="4" t="inlineStr"/>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>

</xml_diff>